<commit_message>
Modified requirement.txt to inlcude pandas and openxyl
</commit_message>
<xml_diff>
--- a/data/DevSec_study_plan.xlsx
+++ b/data/DevSec_study_plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/justin/Desktop/Justin/PycharmProjects/ansible_dev/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{413A58CF-F02F-654C-840E-2EB6C477E35C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13FA93CC-EEDF-B04D-976F-4BD453987EF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="880" windowWidth="36000" windowHeight="21540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15040" yWindow="-21100" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ACI_CONTRACTS" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="60">
   <si>
     <t>CONSUMED_EPG</t>
   </si>
@@ -76,9 +76,6 @@
     <t>INCLUDED IN VZANY DEFAULT RULE</t>
   </si>
   <si>
-    <t>NOTES</t>
-  </si>
-  <si>
     <t>EPG_L3OUT</t>
   </si>
   <si>
@@ -118,9 +115,6 @@
     <t>Yes</t>
   </si>
   <si>
-    <t>DaVinci Robots 151.211.171.2 &amp; 151.211.164.8 to RFL-INTUITIVE 151.211.211.129  - MSMQ - Microsoft Message Queue</t>
-  </si>
-  <si>
     <t>EPG_151.211.208.0</t>
   </si>
   <si>
@@ -136,9 +130,6 @@
     <t>TCP_1434_FLT</t>
   </si>
   <si>
-    <t>RFL-INTUITIVE 151.211.211.129 to SQL Database ,SQL Cluster IP - 151.211.208.87, SQL Instance (SQL-CLIN01-02\INST01) IP: 151.211.209.15</t>
-  </si>
-  <si>
     <t>VZANY</t>
   </si>
   <si>
@@ -187,9 +178,6 @@
     <t>TCP_8888_FLT</t>
   </si>
   <si>
-    <t>DaVinci Robots 151.211.171.2 &amp; 151.211.164.8 to RFL-INTUITIVE 151.211.211.129 - Application Updates</t>
-  </si>
-  <si>
     <t>EPG_DCF</t>
   </si>
   <si>
@@ -208,14 +196,17 @@
     <t>Justin</t>
   </si>
   <si>
-    <t>Created by Ansible</t>
+    <t>STATUS</t>
+  </si>
+  <si>
+    <t>Done</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -227,6 +218,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -264,9 +261,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -590,7 +590,7 @@
     <col min="16" max="16" width="8" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="10.83203125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="28.5" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="110" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="6.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.2">
@@ -648,40 +648,40 @@
       <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
-        <v>18</v>
+      <c r="S1" s="2" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" t="s">
         <v>33</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" t="s">
+      <c r="G2" t="s">
         <v>35</v>
       </c>
-      <c r="E2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G2" t="s">
-        <v>37</v>
-      </c>
       <c r="I2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="J2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K2" t="s">
         <v>26</v>
-      </c>
-      <c r="K2" t="s">
-        <v>27</v>
       </c>
       <c r="L2">
         <v>1434</v>
@@ -690,54 +690,54 @@
         <v>1434</v>
       </c>
       <c r="N2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O2" t="s">
         <v>28</v>
       </c>
-      <c r="O2" t="s">
+      <c r="Q2" t="s">
         <v>29</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>30</v>
       </c>
-      <c r="R2" t="s">
-        <v>31</v>
-      </c>
       <c r="S2" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" t="s">
         <v>39</v>
       </c>
-      <c r="B3" t="s">
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
         <v>40</v>
       </c>
-      <c r="C3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="G3" t="s">
         <v>42</v>
       </c>
-      <c r="E3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>43</v>
       </c>
-      <c r="G3" t="s">
-        <v>45</v>
-      </c>
-      <c r="H3" t="s">
-        <v>46</v>
-      </c>
       <c r="I3" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="J3" t="s">
+        <v>25</v>
+      </c>
+      <c r="K3" t="s">
         <v>26</v>
-      </c>
-      <c r="K3" t="s">
-        <v>27</v>
       </c>
       <c r="L3">
         <v>445</v>
@@ -746,45 +746,45 @@
         <v>445</v>
       </c>
       <c r="N3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="P3" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" t="s">
         <v>39</v>
       </c>
-      <c r="B4" t="s">
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
         <v>40</v>
       </c>
-      <c r="C4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" t="s">
-        <v>43</v>
-      </c>
       <c r="G4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="H4" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="I4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="J4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K4" t="s">
         <v>26</v>
-      </c>
-      <c r="K4" t="s">
-        <v>27</v>
       </c>
       <c r="L4">
         <v>443</v>
@@ -793,42 +793,42 @@
         <v>443</v>
       </c>
       <c r="N4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="P4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
         <v>19</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>20</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>21</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>22</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>23</v>
       </c>
-      <c r="F5" t="s">
-        <v>24</v>
-      </c>
       <c r="G5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="I5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J5" t="s">
+        <v>25</v>
+      </c>
+      <c r="K5" t="s">
         <v>26</v>
-      </c>
-      <c r="K5" t="s">
-        <v>27</v>
       </c>
       <c r="L5">
         <v>135</v>
@@ -837,51 +837,51 @@
         <v>135</v>
       </c>
       <c r="N5" t="s">
+        <v>27</v>
+      </c>
+      <c r="O5" t="s">
         <v>28</v>
       </c>
-      <c r="O5" t="s">
+      <c r="Q5" t="s">
         <v>29</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="R5" t="s">
         <v>30</v>
       </c>
-      <c r="R5" t="s">
-        <v>31</v>
-      </c>
       <c r="S5" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" t="s">
         <v>51</v>
       </c>
-      <c r="B6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" t="s">
-        <v>52</v>
-      </c>
-      <c r="D6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" t="s">
-        <v>53</v>
-      </c>
-      <c r="G6" t="s">
-        <v>54</v>
-      </c>
       <c r="I6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="J6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K6" t="s">
         <v>26</v>
-      </c>
-      <c r="K6" t="s">
-        <v>27</v>
       </c>
       <c r="L6">
         <v>8888</v>
@@ -890,54 +890,54 @@
         <v>8888</v>
       </c>
       <c r="N6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O6" t="s">
         <v>28</v>
       </c>
-      <c r="O6" t="s">
+      <c r="Q6" t="s">
         <v>29</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="R6" t="s">
         <v>30</v>
       </c>
-      <c r="R6" t="s">
-        <v>31</v>
-      </c>
       <c r="S6" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C7" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D7" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F7" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="G7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="H7" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="I7" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="J7" t="s">
+        <v>25</v>
+      </c>
+      <c r="K7" t="s">
         <v>26</v>
-      </c>
-      <c r="K7" t="s">
-        <v>27</v>
       </c>
       <c r="L7">
         <v>445</v>
@@ -946,42 +946,42 @@
         <v>445</v>
       </c>
       <c r="N7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="P7" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" t="s">
         <v>22</v>
       </c>
-      <c r="E8" t="s">
-        <v>23</v>
-      </c>
       <c r="F8" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I8" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="J8" t="s">
+        <v>25</v>
+      </c>
+      <c r="K8" t="s">
         <v>26</v>
-      </c>
-      <c r="K8" t="s">
-        <v>27</v>
       </c>
       <c r="L8">
         <v>8888</v>
@@ -990,51 +990,51 @@
         <v>8888</v>
       </c>
       <c r="N8" t="s">
+        <v>27</v>
+      </c>
+      <c r="O8" t="s">
         <v>28</v>
       </c>
-      <c r="O8" t="s">
-        <v>29</v>
-      </c>
       <c r="Q8" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="R8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="S8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s">
         <v>19</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>20</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>21</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>22</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>23</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>24</v>
       </c>
-      <c r="G9" t="s">
+      <c r="I9" t="s">
+        <v>24</v>
+      </c>
+      <c r="J9" t="s">
         <v>25</v>
       </c>
-      <c r="I9" t="s">
-        <v>25</v>
-      </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>26</v>
-      </c>
-      <c r="K9" t="s">
-        <v>27</v>
       </c>
       <c r="L9">
         <v>2101</v>
@@ -1043,19 +1043,16 @@
         <v>2101</v>
       </c>
       <c r="N9" t="s">
+        <v>27</v>
+      </c>
+      <c r="O9" t="s">
         <v>28</v>
       </c>
-      <c r="O9" t="s">
+      <c r="Q9" t="s">
         <v>29</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="R9" t="s">
         <v>30</v>
-      </c>
-      <c r="R9" t="s">
-        <v>31</v>
-      </c>
-      <c r="S9" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>